<commit_message>
Add database ddl patches 19.09.2025
</commit_message>
<xml_diff>
--- a/1. Database Design/Java24 NguyenHuuThanh Database Design.xlsx
+++ b/1. Database Design/Java24 NguyenHuuThanh Database Design.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java24\3.Database\1. DatabaseDesign\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java24\3.Database\1. Database Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24EEE64A-73A5-47F6-A933-84D412ECA499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65C86153-24AE-4266-809C-D02F5ED3F45E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="B1. Mô hình quan niệm" sheetId="1" r:id="rId1"/>
@@ -1292,7 +1292,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="367">
   <si>
     <t>ChucVu</t>
   </si>
@@ -2055,12 +2055,6 @@
     <t>T23_CART</t>
   </si>
   <si>
-    <t>T23_SHOPPING_CART</t>
-  </si>
-  <si>
-    <t>T24_CART_LATER_ON</t>
-  </si>
-  <si>
     <t>C01_ITEM_ID</t>
   </si>
   <si>
@@ -2130,9 +2124,6 @@
     <t>C23_CART_ID</t>
   </si>
   <si>
-    <t>C24_CUSTOMER_ID</t>
-  </si>
-  <si>
     <t>C01_ITEM_NAME</t>
   </si>
   <si>
@@ -2193,18 +2184,12 @@
     <t>C20_ROLE_NAME</t>
   </si>
   <si>
-    <t>C21_ROLE</t>
-  </si>
-  <si>
     <t>C22_TAX_IN_PERCENT</t>
   </si>
   <si>
     <t>C23_CUSTOMER_ID</t>
   </si>
   <si>
-    <t>C23_ITEM_ID</t>
-  </si>
-  <si>
     <t>C24_ITEM_ID</t>
   </si>
   <si>
@@ -2259,9 +2244,6 @@
     <t>C23_DATE_CREATED</t>
   </si>
   <si>
-    <t>C23_AMOUNT</t>
-  </si>
-  <si>
     <t>C24_AMOUNT</t>
   </si>
   <si>
@@ -2301,9 +2283,6 @@
     <t>C22_DATE_SUBMIT</t>
   </si>
   <si>
-    <t>C23_DATE_ADDING</t>
-  </si>
-  <si>
     <t>C05_PROVIDER_ID</t>
   </si>
   <si>
@@ -2326,9 +2305,6 @@
   </si>
   <si>
     <t>C22_DATE_FROM</t>
-  </si>
-  <si>
-    <t>C23_DATE_REMOVING</t>
   </si>
   <si>
     <t>C09_EMPLOYEE_ID</t>
@@ -2746,24 +2722,45 @@
       <t>) khác, bảng tham chiếu sẽ cần phải có nhiều hơn 1 column làm khóa ngoại</t>
     </r>
   </si>
+  <si>
+    <t>C21_ROLE_ID</t>
+  </si>
+  <si>
+    <t>T24_SHOPPING_CART</t>
+  </si>
+  <si>
+    <t>C24_CART_ID</t>
+  </si>
+  <si>
+    <t>C24_DATE_ADDING</t>
+  </si>
+  <si>
+    <t>C24_DATE_REMOVING</t>
+  </si>
+  <si>
+    <t>T25_CART_LATER_ON</t>
+  </si>
+  <si>
+    <t>C25_CUSTOMER_ID</t>
+  </si>
+  <si>
+    <t>C25_ITEM_ID</t>
+  </si>
+  <si>
+    <t>C25_AMOUNT</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
@@ -3041,44 +3038,47 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3087,106 +3087,103 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4794,21 +4791,21 @@
     </row>
     <row r="26" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B26" s="7" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="C26" s="7"/>
       <c r="D26" s="7"/>
     </row>
     <row r="27" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B27" s="7" t="s">
-        <v>357</v>
+        <v>349</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
     </row>
     <row r="28" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B28" s="7" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
@@ -4829,7 +4826,7 @@
     </row>
     <row r="31" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B31" s="7" t="s">
-        <v>359</v>
+        <v>351</v>
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
@@ -5570,21 +5567,21 @@
     </row>
     <row r="26" spans="2:17" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="7" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="C26" s="7"/>
       <c r="D26" s="7"/>
     </row>
     <row r="27" spans="2:17" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="7" t="s">
-        <v>357</v>
+        <v>349</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
     </row>
     <row r="28" spans="2:17" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="7" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
@@ -5605,7 +5602,7 @@
     </row>
     <row r="31" spans="2:17" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="7" t="s">
-        <v>359</v>
+        <v>351</v>
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
@@ -5711,7 +5708,7 @@
         <v>155</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
     </row>
     <row r="40" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -5738,7 +5735,7 @@
     </row>
     <row r="44" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B44" s="7" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
     </row>
     <row r="45" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -5753,7 +5750,7 @@
     </row>
     <row r="47" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B47" s="17" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
     </row>
     <row r="48" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -5924,7 +5921,7 @@
     <row r="60" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="61" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B61" s="7" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
     </row>
     <row r="62" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -5940,7 +5937,7 @@
     </row>
     <row r="65" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B65" s="7" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="G65" s="7" t="s">
         <v>188</v>
@@ -6565,281 +6562,281 @@
         <v>236</v>
       </c>
       <c r="Y5" s="2" t="s">
-        <v>237</v>
+        <v>359</v>
       </c>
       <c r="Z5" s="2" t="s">
-        <v>238</v>
+        <v>363</v>
       </c>
     </row>
     <row r="6" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="D6" s="27" t="s">
         <v>239</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="E6" s="11" t="s">
         <v>240</v>
       </c>
-      <c r="D6" s="27" t="s">
+      <c r="F6" s="27" t="s">
         <v>241</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="G6" s="11" t="s">
         <v>242</v>
       </c>
-      <c r="F6" s="27" t="s">
+      <c r="H6" s="11" t="s">
         <v>243</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="I6" s="11" t="s">
         <v>244</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="J6" s="11" t="s">
         <v>245</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="K6" s="11" t="s">
         <v>246</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="L6" s="11" t="s">
         <v>247</v>
       </c>
-      <c r="K6" s="11" t="s">
+      <c r="M6" s="27" t="s">
         <v>248</v>
       </c>
-      <c r="L6" s="11" t="s">
+      <c r="N6" s="11" t="s">
         <v>249</v>
       </c>
-      <c r="M6" s="27" t="s">
+      <c r="O6" s="27" t="s">
         <v>250</v>
       </c>
-      <c r="N6" s="11" t="s">
+      <c r="P6" s="11" t="s">
         <v>251</v>
       </c>
-      <c r="O6" s="27" t="s">
+      <c r="Q6" s="11" t="s">
         <v>252</v>
       </c>
-      <c r="P6" s="11" t="s">
+      <c r="R6" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="Q6" s="11" t="s">
+      <c r="S6" s="11" t="s">
         <v>254</v>
       </c>
-      <c r="R6" s="11" t="s">
+      <c r="T6" s="11" t="s">
         <v>255</v>
       </c>
-      <c r="S6" s="11" t="s">
+      <c r="U6" s="11" t="s">
         <v>256</v>
       </c>
-      <c r="T6" s="11" t="s">
+      <c r="V6" s="27" t="s">
         <v>257</v>
       </c>
-      <c r="U6" s="11" t="s">
+      <c r="W6" s="11" t="s">
         <v>258</v>
       </c>
-      <c r="V6" s="27" t="s">
+      <c r="X6" s="11" t="s">
         <v>259</v>
       </c>
-      <c r="W6" s="11" t="s">
-        <v>260</v>
-      </c>
-      <c r="X6" s="11" t="s">
-        <v>261</v>
-      </c>
       <c r="Y6" s="27" t="s">
-        <v>261</v>
+        <v>360</v>
       </c>
       <c r="Z6" s="27" t="s">
-        <v>262</v>
+        <v>364</v>
       </c>
     </row>
     <row r="7" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="C7" s="31" t="s">
+        <v>261</v>
+      </c>
+      <c r="D7" s="27" t="s">
+        <v>262</v>
+      </c>
+      <c r="E7" s="11" t="s">
         <v>263</v>
       </c>
-      <c r="C7" s="31" t="s">
+      <c r="F7" s="27" t="s">
         <v>264</v>
       </c>
-      <c r="D7" s="27" t="s">
+      <c r="G7" s="14" t="s">
         <v>265</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="H7" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="F7" s="27" t="s">
+      <c r="I7" s="14" t="s">
         <v>267</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="J7" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="K7" s="28" t="s">
         <v>269</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="L7" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="M7" s="27" t="s">
         <v>271</v>
       </c>
-      <c r="K7" s="28" t="s">
+      <c r="N7" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="L7" s="3" t="s">
+      <c r="O7" s="27" t="s">
         <v>273</v>
       </c>
-      <c r="M7" s="27" t="s">
+      <c r="P7" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="N7" s="3" t="s">
+      <c r="Q7" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="O7" s="27" t="s">
+      <c r="R7" s="11" t="s">
         <v>276</v>
       </c>
-      <c r="P7" s="3" t="s">
+      <c r="S7" s="28" t="s">
         <v>277</v>
       </c>
-      <c r="Q7" s="3" t="s">
+      <c r="T7" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="R7" s="11" t="s">
+      <c r="U7" s="26" t="s">
         <v>279</v>
       </c>
-      <c r="S7" s="28" t="s">
+      <c r="V7" s="27" t="s">
+        <v>358</v>
+      </c>
+      <c r="W7" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="T7" s="3" t="s">
+      <c r="X7" s="28" t="s">
         <v>281</v>
       </c>
-      <c r="U7" s="26" t="s">
+      <c r="Y7" s="27" t="s">
         <v>282</v>
       </c>
-      <c r="V7" s="27" t="s">
-        <v>283</v>
-      </c>
-      <c r="W7" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="X7" s="28" t="s">
-        <v>285</v>
-      </c>
-      <c r="Y7" s="27" t="s">
-        <v>286</v>
-      </c>
       <c r="Z7" s="27" t="s">
-        <v>287</v>
+        <v>365</v>
       </c>
     </row>
     <row r="8" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="28" t="s">
+        <v>283</v>
+      </c>
+      <c r="C8" s="31" t="s">
+        <v>284</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="G8" s="14" t="s">
         <v>288</v>
       </c>
-      <c r="C8" s="31" t="s">
+      <c r="H8" s="3" t="s">
         <v>289</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>290</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="G8" s="14" t="s">
-        <v>293</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>294</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="28" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="L8" s="3"/>
       <c r="M8" s="3" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="N8" s="3"/>
       <c r="O8" s="28" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="R8" s="3"/>
       <c r="S8" s="3" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="U8" s="3"/>
       <c r="V8" s="3"/>
       <c r="W8" s="3" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="X8" s="3" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="Y8" s="3" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="Z8" s="3" t="s">
-        <v>306</v>
+        <v>366</v>
       </c>
     </row>
     <row r="9" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="3" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="28" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="K9" s="13" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
       <c r="O9" s="3" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="Q9" s="3" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="R9" s="3"/>
       <c r="S9" s="3" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="T9" s="3" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="U9" s="3"/>
       <c r="V9" s="3"/>
       <c r="W9" s="3" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="X9" s="3"/>
       <c r="Y9" s="3" t="s">
-        <v>319</v>
+        <v>361</v>
       </c>
       <c r="Z9" s="3"/>
     </row>
@@ -6849,42 +6846,42 @@
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" s="28" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="28" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="K10" s="14" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="L10" s="13"/>
       <c r="M10" s="13"/>
       <c r="N10" s="13"/>
       <c r="O10" s="13"/>
       <c r="P10" s="3" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="Q10" s="3" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="R10" s="3"/>
       <c r="S10" s="3" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="T10" s="3" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="U10" s="3"/>
       <c r="V10" s="3"/>
       <c r="W10" s="3" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="X10" s="3"/>
       <c r="Y10" s="3" t="s">
-        <v>328</v>
+        <v>362</v>
       </c>
       <c r="Z10" s="3"/>
     </row>
@@ -6898,7 +6895,7 @@
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="28" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="K11" s="13"/>
       <c r="L11" s="5"/>
@@ -6906,20 +6903,20 @@
       <c r="N11" s="5"/>
       <c r="O11" s="5"/>
       <c r="P11" s="3" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="Q11" s="3" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="R11" s="3"/>
       <c r="S11" s="3"/>
       <c r="T11" s="3" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="U11" s="3"/>
       <c r="V11" s="3"/>
       <c r="W11" s="3" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="X11" s="3"/>
       <c r="Y11" s="3"/>
@@ -6941,10 +6938,10 @@
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="Q12" s="3" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="R12" s="3"/>
       <c r="S12" s="3"/>
@@ -6952,7 +6949,7 @@
       <c r="U12" s="3"/>
       <c r="V12" s="3"/>
       <c r="W12" s="28" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="Y12" s="3"/>
       <c r="Z12" s="3"/>
@@ -6974,7 +6971,7 @@
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
       <c r="Q13" s="28" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="R13" s="13"/>
       <c r="S13" s="3"/>
@@ -7151,30 +7148,30 @@
     <row r="20" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="21" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
     </row>
     <row r="22" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="7" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="V22" s="7"/>
     </row>
     <row r="23" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="32" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="V23" s="7"/>
     </row>
     <row r="24" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="7" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="V24" s="7"/>
     </row>
     <row r="25" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="7" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="V25" s="7"/>
     </row>
@@ -7182,13 +7179,13 @@
       <c r="B26" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="C26" s="33" t="s">
-        <v>342</v>
-      </c>
-      <c r="D26" s="34"/>
-      <c r="E26" s="35"/>
-      <c r="F26" s="35"/>
-      <c r="G26" s="35"/>
+      <c r="C26" s="47" t="s">
+        <v>334</v>
+      </c>
+      <c r="D26" s="48"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="33"/>
       <c r="H26" s="6"/>
       <c r="I26" s="6"/>
       <c r="K26" s="2" t="s">
@@ -7196,27 +7193,27 @@
       </c>
     </row>
     <row r="27" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="36" t="s">
-        <v>240</v>
-      </c>
-      <c r="C27" s="37" t="s">
-        <v>264</v>
-      </c>
-      <c r="D27" s="37" t="s">
-        <v>289</v>
-      </c>
-      <c r="E27" s="37"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="37"/>
-      <c r="H27" s="38" t="s">
-        <v>308</v>
-      </c>
-      <c r="I27" s="39"/>
-      <c r="K27" s="36" t="s">
-        <v>239</v>
-      </c>
-      <c r="L27" s="36" t="s">
-        <v>240</v>
+      <c r="B27" s="34" t="s">
+        <v>238</v>
+      </c>
+      <c r="C27" s="35" t="s">
+        <v>261</v>
+      </c>
+      <c r="D27" s="35" t="s">
+        <v>284</v>
+      </c>
+      <c r="E27" s="35"/>
+      <c r="F27" s="35"/>
+      <c r="G27" s="35"/>
+      <c r="H27" s="36" t="s">
+        <v>302</v>
+      </c>
+      <c r="I27" s="37"/>
+      <c r="K27" s="34" t="s">
+        <v>237</v>
+      </c>
+      <c r="L27" s="34" t="s">
+        <v>238</v>
       </c>
       <c r="M27" s="29"/>
       <c r="N27" s="29"/>
@@ -7226,21 +7223,21 @@
       <c r="B28" s="7">
         <v>1</v>
       </c>
-      <c r="C28" s="40" t="s">
+      <c r="C28" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="D28" s="40">
+      <c r="D28" s="38">
         <v>0</v>
       </c>
-      <c r="E28" s="40"/>
-      <c r="F28" s="40"/>
-      <c r="G28" s="40"/>
-      <c r="H28" s="40" t="s">
-        <v>343</v>
-      </c>
-      <c r="I28" s="40"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="38" t="s">
+        <v>335</v>
+      </c>
+      <c r="I28" s="38"/>
       <c r="K28" s="7" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="L28" s="7">
         <v>1</v>
@@ -7253,19 +7250,19 @@
       <c r="B29" s="7">
         <v>2</v>
       </c>
-      <c r="C29" s="40" t="s">
+      <c r="C29" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="D29" s="40">
+      <c r="D29" s="38">
         <v>0</v>
       </c>
-      <c r="E29" s="40"/>
-      <c r="F29" s="40"/>
-      <c r="G29" s="40"/>
-      <c r="H29" s="40"/>
-      <c r="I29" s="40"/>
+      <c r="E29" s="38"/>
+      <c r="F29" s="38"/>
+      <c r="G29" s="38"/>
+      <c r="H29" s="38"/>
+      <c r="I29" s="38"/>
       <c r="K29" s="7" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="L29" s="7">
         <v>1</v>
@@ -7278,19 +7275,19 @@
       <c r="B30" s="7">
         <v>3</v>
       </c>
-      <c r="C30" s="40" t="s">
+      <c r="C30" s="38" t="s">
         <v>133</v>
       </c>
-      <c r="D30" s="40">
+      <c r="D30" s="38">
         <v>0</v>
       </c>
-      <c r="E30" s="40"/>
-      <c r="F30" s="40"/>
-      <c r="G30" s="40"/>
-      <c r="H30" s="40"/>
-      <c r="I30" s="40"/>
+      <c r="E30" s="38"/>
+      <c r="F30" s="38"/>
+      <c r="G30" s="38"/>
+      <c r="H30" s="38"/>
+      <c r="I30" s="38"/>
       <c r="K30" s="7" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="L30" s="7">
         <v>7</v>
@@ -7303,33 +7300,33 @@
       <c r="B31" s="7">
         <v>4</v>
       </c>
-      <c r="C31" s="40" t="s">
-        <v>347</v>
-      </c>
-      <c r="D31" s="40">
+      <c r="C31" s="38" t="s">
+        <v>339</v>
+      </c>
+      <c r="D31" s="38">
         <v>0</v>
       </c>
-      <c r="E31" s="40"/>
-      <c r="F31" s="40"/>
-      <c r="G31" s="40"/>
-      <c r="H31" s="40"/>
-      <c r="I31" s="40"/>
+      <c r="E31" s="38"/>
+      <c r="F31" s="38"/>
+      <c r="G31" s="38"/>
+      <c r="H31" s="38"/>
+      <c r="I31" s="38"/>
     </row>
     <row r="32" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="7">
         <v>5</v>
       </c>
-      <c r="C32" s="40" t="s">
-        <v>348</v>
-      </c>
-      <c r="D32" s="40">
+      <c r="C32" s="38" t="s">
+        <v>340</v>
+      </c>
+      <c r="D32" s="38">
         <v>0</v>
       </c>
-      <c r="E32" s="40"/>
-      <c r="F32" s="40"/>
-      <c r="G32" s="40"/>
-      <c r="H32" s="40"/>
-      <c r="I32" s="40"/>
+      <c r="E32" s="38"/>
+      <c r="F32" s="38"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="38"/>
+      <c r="I32" s="38"/>
       <c r="U32" s="9"/>
       <c r="V32" s="9"/>
     </row>
@@ -7337,19 +7334,19 @@
       <c r="B33" s="7">
         <v>6</v>
       </c>
-      <c r="C33" s="40" t="s">
+      <c r="C33" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="D33" s="40">
+      <c r="D33" s="38">
         <v>1</v>
       </c>
-      <c r="E33" s="40"/>
-      <c r="F33" s="40"/>
-      <c r="G33" s="40"/>
-      <c r="H33" s="40" t="s">
-        <v>349</v>
-      </c>
-      <c r="I33" s="40"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="38" t="s">
+        <v>341</v>
+      </c>
+      <c r="I33" s="38"/>
       <c r="S33" s="9"/>
       <c r="T33" s="9"/>
     </row>
@@ -7357,17 +7354,17 @@
       <c r="B34" s="7">
         <v>7</v>
       </c>
-      <c r="C34" s="40" t="s">
+      <c r="C34" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="D34" s="40">
+      <c r="D34" s="38">
         <v>1</v>
       </c>
-      <c r="E34" s="40"/>
-      <c r="F34" s="40"/>
-      <c r="G34" s="40"/>
-      <c r="H34" s="40"/>
-      <c r="I34" s="40"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="38"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="38"/>
+      <c r="I34" s="38"/>
       <c r="S34" s="9"/>
       <c r="T34" s="9"/>
     </row>
@@ -7375,66 +7372,66 @@
       <c r="B35" s="7">
         <v>8</v>
       </c>
-      <c r="C35" s="40" t="s">
+      <c r="C35" s="38" t="s">
         <v>133</v>
       </c>
-      <c r="D35" s="40">
+      <c r="D35" s="38">
         <v>1</v>
       </c>
-      <c r="E35" s="40"/>
-      <c r="F35" s="40"/>
-      <c r="G35" s="40"/>
-      <c r="H35" s="40"/>
-      <c r="I35" s="40"/>
+      <c r="E35" s="38"/>
+      <c r="F35" s="38"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="38"/>
+      <c r="I35" s="38"/>
       <c r="T35" s="9"/>
     </row>
     <row r="36" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="7">
         <v>9</v>
       </c>
-      <c r="C36" s="40" t="s">
-        <v>347</v>
-      </c>
-      <c r="D36" s="40">
+      <c r="C36" s="38" t="s">
+        <v>339</v>
+      </c>
+      <c r="D36" s="38">
         <v>1</v>
       </c>
-      <c r="E36" s="40"/>
-      <c r="F36" s="40"/>
-      <c r="G36" s="40"/>
-      <c r="H36" s="40"/>
-      <c r="I36" s="40"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="38"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="38"/>
+      <c r="I36" s="38"/>
       <c r="T36" s="9"/>
     </row>
     <row r="37" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="7">
         <v>10</v>
       </c>
-      <c r="C37" s="40" t="s">
-        <v>348</v>
-      </c>
-      <c r="D37" s="40">
+      <c r="C37" s="38" t="s">
+        <v>340</v>
+      </c>
+      <c r="D37" s="38">
         <v>1</v>
       </c>
-      <c r="E37" s="40"/>
-      <c r="F37" s="40"/>
-      <c r="G37" s="40"/>
-      <c r="H37" s="40"/>
-      <c r="I37" s="40"/>
+      <c r="E37" s="38"/>
+      <c r="F37" s="38"/>
+      <c r="G37" s="38"/>
+      <c r="H37" s="38"/>
+      <c r="I37" s="38"/>
     </row>
     <row r="38" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>145</v>
       </c>
       <c r="B38" s="7"/>
-      <c r="C38" s="41" t="s">
-        <v>348</v>
-      </c>
-      <c r="D38" s="41">
+      <c r="C38" s="39" t="s">
+        <v>340</v>
+      </c>
+      <c r="D38" s="39">
         <v>1</v>
       </c>
-      <c r="E38" s="41"/>
-      <c r="F38" s="41"/>
-      <c r="G38" s="41"/>
+      <c r="E38" s="39"/>
+      <c r="F38" s="39"/>
+      <c r="G38" s="39"/>
       <c r="H38" s="7"/>
       <c r="I38" s="7"/>
     </row>
@@ -7450,7 +7447,7 @@
     </row>
     <row r="40" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="7" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="C40" s="17"/>
       <c r="D40" s="17"/>
@@ -7486,59 +7483,59 @@
       <c r="I42" s="9"/>
     </row>
     <row r="43" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="36" t="s">
-        <v>246</v>
-      </c>
-      <c r="C43" s="37" t="s">
-        <v>270</v>
+      <c r="B43" s="34" t="s">
+        <v>244</v>
+      </c>
+      <c r="C43" s="35" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="44" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="42" t="s">
-        <v>351</v>
+      <c r="B44" s="40" t="s">
+        <v>343</v>
       </c>
       <c r="C44" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B45" s="42" t="s">
-        <v>352</v>
+      <c r="B45" s="40" t="s">
+        <v>344</v>
       </c>
       <c r="C45" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B46" s="42" t="s">
-        <v>353</v>
+      <c r="B46" s="40" t="s">
+        <v>345</v>
       </c>
       <c r="C46" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B47" s="42" t="s">
-        <v>354</v>
+      <c r="B47" s="40" t="s">
+        <v>346</v>
       </c>
       <c r="C47" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B48" s="42" t="s">
-        <v>355</v>
+      <c r="B48" s="40" t="s">
+        <v>347</v>
       </c>
       <c r="C48" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="49" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B49" s="43"/>
+      <c r="B49" s="41"/>
     </row>
     <row r="50" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B50" s="44"/>
-      <c r="J50" s="45"/>
+      <c r="B50" s="42"/>
+      <c r="J50" s="43"/>
     </row>
     <row r="51" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="L51" s="7"/>
@@ -7554,21 +7551,21 @@
     </row>
     <row r="53" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="54" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="L54" s="43"/>
-      <c r="M54" s="43"/>
-      <c r="N54" s="43"/>
-      <c r="O54" s="43"/>
+      <c r="L54" s="41"/>
+      <c r="M54" s="41"/>
+      <c r="N54" s="41"/>
+      <c r="O54" s="41"/>
     </row>
     <row r="55" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B55" s="43"/>
+      <c r="B55" s="41"/>
     </row>
     <row r="56" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B56" s="44"/>
-      <c r="L56" s="44"/>
-      <c r="M56" s="44"/>
-      <c r="N56" s="44"/>
-      <c r="O56" s="44"/>
-      <c r="P56" s="46"/>
+      <c r="B56" s="42"/>
+      <c r="L56" s="42"/>
+      <c r="M56" s="42"/>
+      <c r="N56" s="42"/>
+      <c r="O56" s="42"/>
+      <c r="P56" s="44"/>
     </row>
     <row r="57" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="58" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -7594,16 +7591,16 @@
     </row>
     <row r="67" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="68" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B68" s="43"/>
-      <c r="L68" s="43"/>
-      <c r="M68" s="43"/>
-      <c r="N68" s="43"/>
-      <c r="O68" s="43"/>
+      <c r="B68" s="41"/>
+      <c r="L68" s="41"/>
+      <c r="M68" s="41"/>
+      <c r="N68" s="41"/>
+      <c r="O68" s="41"/>
     </row>
     <row r="69" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B69" s="44"/>
-      <c r="H69" s="47"/>
-      <c r="I69" s="47"/>
+      <c r="B69" s="42"/>
+      <c r="H69" s="45"/>
+      <c r="I69" s="45"/>
       <c r="L69" s="9"/>
       <c r="M69" s="9"/>
       <c r="N69" s="9"/>
@@ -7611,11 +7608,11 @@
       <c r="P69" s="9"/>
     </row>
     <row r="70" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="L70" s="47"/>
-      <c r="M70" s="47"/>
-      <c r="N70" s="47"/>
-      <c r="O70" s="47"/>
-      <c r="P70" s="47"/>
+      <c r="L70" s="45"/>
+      <c r="M70" s="45"/>
+      <c r="N70" s="45"/>
+      <c r="O70" s="45"/>
+      <c r="P70" s="45"/>
     </row>
     <row r="71" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C71" s="8"/>
@@ -7627,14 +7624,14 @@
     <row r="72" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="73" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="74" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B74" s="43"/>
+      <c r="B74" s="41"/>
       <c r="J74" s="9"/>
     </row>
     <row r="75" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B75" s="44"/>
-      <c r="H75" s="48"/>
-      <c r="I75" s="48"/>
-      <c r="J75" s="47"/>
+      <c r="B75" s="42"/>
+      <c r="H75" s="46"/>
+      <c r="I75" s="46"/>
+      <c r="J75" s="45"/>
     </row>
     <row r="76" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="77" spans="2:16" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -7663,7 +7660,7 @@
       <c r="F85" s="3"/>
       <c r="G85" s="3"/>
       <c r="H85" s="13"/>
-      <c r="I85" s="47"/>
+      <c r="I85" s="45"/>
     </row>
     <row r="86" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="87" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>